<commit_message>
fix data on dataset
</commit_message>
<xml_diff>
--- a/cis_azure_vmware.xlsx
+++ b/cis_azure_vmware.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Azure CIS" sheetId="1" state="visible" r:id="rId3"/>
@@ -101,66 +101,66 @@
     <t xml:space="preserve">false</t>
   </si>
   <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure 'FTP state' is set to 'FTPS only' or 'Disabled'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By default, App Service supports deployment over FTP. If FTP is essential for a deployment workflow, FTPS should be enforced for all function apps. If FTPS is not explicitly required, the recommended setting is Disabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTP is an unencrypted network protocol that transmits data—including passwords—in clear text. The use of this protocol can lead to both data and credential compromise and can present opportunities for exfiltration, persistence, and lateral movement. HINT: Ensure that "FtpsOnly" or "Disabled" is returned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deployment workflows that rely on FTP or FTPS rather than WebDeploy or HTTPS endpoints may be affected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">az functionapp list // az functionapp show --resource-group &lt;resource-group-name&gt; --name &lt;functionapp-name&gt; --query siteConfig.ftpsState</t>
+  </si>
+  <si>
+    <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --ftps-state &lt;FtpsOnly|Disabled&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ftpsState</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FtpsOnly | Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure 'HTTP version' is set to '2.0' (if in use) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodically, newer versions are released for HTTP, either due to security flaws or to include additional functionalities. Using the latest HTTP version allows apps to take advantage of security fixes, if any, and/or new functionalities of the newer version.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newer versions may contain security enhancements and additional functionalities. Using the latest version is recommended in order to take advantage of enhancements and new capabilities. With each software installation, organizations need to determine if a given update meets their requirements. They must also verify the compatibility and support provided for any additional software against the update revision that is selected. HTTP 2.0 has additional performance improvements for the head-of-line blocking problem of the old HTTP version, header compression, and request prioritization. HTTP 2.0 no longer supports HTTP 1.1's chunked transfer encoding mechanism, as it provides its own, more efficient mechanisms for data streaming. HINT: Ensure that true is returned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most modern browsers support the HTTP/2 protocol over TLS only, while non-encrypted traffic continues to use HTTP/1.1. To ensure that client browsers connect to your app with HTTP/2, either purchase an App Service Certificate for your app's custom domain or bind a third-party certificate. NOTE: HTTP/2 cannot be used in tandem with mutual authentication or client certificates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">az functionapp list // az functionapp config show --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --query http20Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;appname&gt; --http20-enabled true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">siteConfig.http20Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
     <t xml:space="preserve">eq</t>
   </si>
   <si>
-    <t xml:space="preserve">2.3.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ensure 'FTP state' is set to 'FTPS only' or 'Disabled'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By default, App Service supports deployment over FTP. If FTP is essential for a deployment workflow, FTPS should be enforced for all function apps. If FTPS is not explicitly required, the recommended setting is Disabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FTP is an unencrypted network protocol that transmits data—including passwords—in clear text. The use of this protocol can lead to both data and credential compromise and can present opportunities for exfiltration, persistence, and lateral movement. HINT: Ensure that "FtpsOnly" or "Disabled" is returned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deployment workflows that rely on FTP or FTPS rather than WebDeploy or HTTPS endpoints may be affected.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">az functionapp list // az functionapp show --resource-group &lt;resource-group-name&gt; --name &lt;functionapp-name&gt; --query siteConfig.ftpsState</t>
-  </si>
-  <si>
-    <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --ftps-state &lt;FtpsOnly|Disabled&gt; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ftpsState</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FtpsOnly | Disabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ensure 'HTTP version' is set to '2.0' (if in use) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Periodically, newer versions are released for HTTP, either due to security flaws or to include additional functionalities. Using the latest HTTP version allows apps to take advantage of security fixes, if any, and/or new functionalities of the newer version.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Newer versions may contain security enhancements and additional functionalities. Using the latest version is recommended in order to take advantage of enhancements and new capabilities. With each software installation, organizations need to determine if a given update meets their requirements. They must also verify the compatibility and support provided for any additional software against the update revision that is selected. HTTP 2.0 has additional performance improvements for the head-of-line blocking problem of the old HTTP version, header compression, and request prioritization. HTTP 2.0 no longer supports HTTP 1.1's chunked transfer encoding mechanism, as it provides its own, more efficient mechanisms for data streaming. HINT: Ensure that true is returned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Most modern browsers support the HTTP/2 protocol over TLS only, while non-encrypted traffic continues to use HTTP/1.1. To ensure that client browsers connect to your app with HTTP/2, either purchase an App Service Certificate for your app's custom domain or bind a third-party certificate. NOTE: HTTP/2 cannot be used in tandem with mutual authentication or client certificates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">az functionapp list // az functionapp config show --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --query http20Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;appname&gt; --http20-enabled true</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http20Enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">true</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.3.6</t>
   </si>
   <si>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --min-tls-version &lt;1.2|1.3&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">minTlsVersion</t>
+    <t xml:space="preserve">siteConfig.minTlsVersion</t>
   </si>
   <si>
     <t xml:space="preserve">1.2</t>
@@ -257,7 +257,7 @@
     <t xml:space="preserve">az functionapp config set --resource-group &lt;resource-group-name&gt; --name &lt;function-app-name&gt; --remote-debugging-enabled false</t>
   </si>
   <si>
-    <t xml:space="preserve">remoteDebuggingEnabled</t>
+    <t xml:space="preserve">siteConfig.remoteDebuggingEnabled</t>
   </si>
   <si>
     <t xml:space="preserve">2.3.10</t>
@@ -410,7 +410,7 @@
     <t xml:space="preserve">az resource update --resource-group &lt;resource-group-name&gt; --name &lt;functionapp-name&gt; --resource-type "Microsoft.Web/sites" --set properties.vnetImagePullEnabled=true --set properties.vnetContentShareEnabled=true</t>
   </si>
   <si>
-    <t xml:space="preserve">vnetRouteAllEnabled</t>
+    <t xml:space="preserve">siteConfig.vnetRouteAllEnabled</t>
   </si>
   <si>
     <t xml:space="preserve">2.3.16</t>
@@ -885,7 +885,7 @@
     <t xml:space="preserve">az network application-gateway list // az network application-gateway show --resource-group &lt;resource-group&gt; --name &lt;application-gateway&gt; --query firewallPolicy.id Ensure a firewall policy id is returned.</t>
   </si>
   <si>
-    <t xml:space="preserve">webApplicationFirewallPolicy</t>
+    <t xml:space="preserve">webApplicationFirewallConfiguration.enabled</t>
   </si>
   <si>
     <t xml:space="preserve">7.11</t>
@@ -957,7 +957,7 @@
     <t xml:space="preserve">az network application-gateway update --resource-group &lt;resource-group&gt; -- name &lt;application-gateway&gt; --http2 Enabled</t>
   </si>
   <si>
-    <t xml:space="preserve">http2Enabled</t>
+    <t xml:space="preserve">enableHttp2</t>
   </si>
   <si>
     <t xml:space="preserve">7.14</t>
@@ -3206,7 +3206,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="57.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="79.8"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="10" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="41.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="37.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="6"/>
@@ -3350,36 +3350,36 @@
         <v>35</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>1</v>
@@ -3391,13 +3391,13 @@
         <v>1</v>
       </c>
       <c r="M4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="O4" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3441,10 +3441,10 @@
         <v>53</v>
       </c>
       <c r="N5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3491,7 +3491,7 @@
         <v>62</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3536,7 +3536,7 @@
         <v>70</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="126.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3583,7 +3583,7 @@
         <v>25</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3627,10 +3627,10 @@
         <v>87</v>
       </c>
       <c r="N9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O9" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3674,10 +3674,10 @@
         <v>95</v>
       </c>
       <c r="N10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O10" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3724,7 +3724,7 @@
         <v>104</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3771,7 +3771,7 @@
         <v>113</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3860,10 +3860,10 @@
         <v>129</v>
       </c>
       <c r="N14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O14" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O14" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3908,7 +3908,7 @@
         <v>136</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3955,7 +3955,7 @@
         <v>145</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4000,7 +4000,7 @@
         <v>154</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4047,7 +4047,7 @@
         <v>161</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="81" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4091,7 +4091,7 @@
         <v>168</v>
       </c>
       <c r="N19" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O19" s="4" t="s">
         <v>26</v>
@@ -4141,7 +4141,7 @@
         <v>176</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4188,7 +4188,7 @@
         <v>182</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4235,7 +4235,7 @@
         <v>188</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4282,7 +4282,7 @@
         <v>194</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4329,7 +4329,7 @@
         <v>201</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4376,7 +4376,7 @@
         <v>208</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4420,7 +4420,7 @@
         <v>214</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4467,7 +4467,7 @@
         <v>220</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4514,7 +4514,7 @@
         <v>226</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4561,7 +4561,7 @@
         <v>232</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4606,7 +4606,7 @@
         <v>240</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4651,7 +4651,7 @@
         <v>248</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4696,7 +4696,7 @@
         <v>256</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4741,7 +4741,7 @@
         <v>261</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4786,7 +4786,7 @@
         <v>266</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4831,7 +4831,7 @@
         <v>271</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="N38" s="4"/>
       <c r="O38" s="4" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5015,7 +5015,7 @@
         <v>303</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5059,10 +5059,10 @@
         <v>311</v>
       </c>
       <c r="N40" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O40" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O40" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5106,10 +5106,10 @@
         <v>319</v>
       </c>
       <c r="N41" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O41" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O41" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="92.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5156,7 +5156,7 @@
         <v>328</v>
       </c>
       <c r="O42" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5203,7 +5203,7 @@
         <v>338</v>
       </c>
       <c r="O43" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5250,7 +5250,7 @@
         <v>338</v>
       </c>
       <c r="O44" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5297,7 +5297,7 @@
         <v>338</v>
       </c>
       <c r="O45" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5344,7 +5344,7 @@
         <v>338</v>
       </c>
       <c r="O46" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5391,7 +5391,7 @@
         <v>338</v>
       </c>
       <c r="O47" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5438,7 +5438,7 @@
         <v>338</v>
       </c>
       <c r="O48" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5485,7 +5485,7 @@
         <v>338</v>
       </c>
       <c r="O49" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5532,7 +5532,7 @@
         <v>338</v>
       </c>
       <c r="O50" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5579,7 +5579,7 @@
         <v>338</v>
       </c>
       <c r="O51" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5626,7 +5626,7 @@
         <v>338</v>
       </c>
       <c r="O52" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5673,7 +5673,7 @@
         <v>338</v>
       </c>
       <c r="O53" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5720,7 +5720,7 @@
         <v>338</v>
       </c>
       <c r="O54" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5904,7 +5904,7 @@
         <v>441</v>
       </c>
       <c r="O58" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5951,7 +5951,7 @@
         <v>457</v>
       </c>
       <c r="O59" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5998,7 +5998,7 @@
         <v>466</v>
       </c>
       <c r="O60" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6042,10 +6042,10 @@
         <v>473</v>
       </c>
       <c r="N61" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O61" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="O61" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -6170,7 +6170,7 @@
         <v>482</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6215,7 +6215,7 @@
         <v>490</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6262,7 +6262,7 @@
         <v>499</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6307,7 +6307,7 @@
         <v>508</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6352,7 +6352,7 @@
         <v>508</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6399,7 +6399,7 @@
         <v>25</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6587,7 +6587,7 @@
         <v>560</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6634,7 +6634,7 @@
         <v>569</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6679,7 +6679,7 @@
         <v>577</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6724,7 +6724,7 @@
         <v>584</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6814,7 +6814,7 @@
         <v>602</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="186.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6859,7 +6859,7 @@
         <v>610</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="186.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6904,7 +6904,7 @@
         <v>617</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6949,7 +6949,7 @@
         <v>624</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6994,7 +6994,7 @@
         <v>632</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7039,7 +7039,7 @@
         <v>641</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7086,7 +7086,7 @@
         <v>649</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7133,7 +7133,7 @@
         <v>658</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="98.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7180,7 +7180,7 @@
         <v>665</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7225,7 +7225,7 @@
         <v>673</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7272,7 +7272,7 @@
         <v>658</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="129" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7319,7 +7319,7 @@
         <v>658</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7364,7 +7364,7 @@
         <v>694</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7409,7 +7409,7 @@
         <v>700</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7454,7 +7454,7 @@
         <v>706</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7499,7 +7499,7 @@
         <v>711</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7544,7 +7544,7 @@
         <v>717</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7591,7 +7591,7 @@
         <v>658</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7638,7 +7638,7 @@
         <v>658</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7685,7 +7685,7 @@
         <v>658</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7732,7 +7732,7 @@
         <v>658</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7779,7 +7779,7 @@
         <v>658</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7826,7 +7826,7 @@
         <v>764</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7873,7 +7873,7 @@
         <v>773</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7920,7 +7920,7 @@
         <v>782</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>